<commit_message>
Integrate player attributes and buff shop
</commit_message>
<xml_diff>
--- a/Config/Luban/Datas/#game.gameEvent.xlsx
+++ b/Config/Luban/Datas/#game.gameEvent.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\AXR_Projects\unity\Anchor\Config\Luban\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09CE75C4-7DE7-40A3-BB4C-268414C77807}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E238230D-6022-4710-B427-7BDD1E32BD15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="37">
   <si>
     <t>##var</t>
   </si>
@@ -40,15 +40,15 @@
     <t>noEffects#format=json</t>
   </si>
   <si>
-    <t>triggerConditions#format=json</t>
+    <t>triggerGreaterOrEqualConditions#format=json</t>
+  </si>
+  <si>
+    <t>triggerLessThanConditions#format=json</t>
   </si>
   <si>
     <t>ratio</t>
   </si>
   <si>
-    <t>cost</t>
-  </si>
-  <si>
     <t>##type</t>
   </si>
   <si>
@@ -82,13 +82,10 @@
     <t>选择N后的属性修改，格式[[属性ID,值]]</t>
   </si>
   <si>
-    <t>触发条件，格式[[属性ID,阈值]]；阈值正负语义由运行时解释</t>
-  </si>
-  <si>
-    <t>Ratio（随机事件的触发概率）</t>
-  </si>
-  <si>
-    <t>Cost（花费）</t>
+    <t>大于等于触发条件，格式[[属性ID,阈值]]；玩家属性 &gt;= 阈值时满足</t>
+  </si>
+  <si>
+    <t>小于触发条件，格式[[属性ID,阈值]]；玩家属性 &lt; 阈值时满足</t>
   </si>
   <si>
     <t>测试事件-愿望增加</t>
@@ -131,13 +128,30 @@
   </si>
   <si>
     <t>[[1009,50]]</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Ratio</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>（随机事件的触发概率）</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -157,6 +171,13 @@
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="4">
@@ -523,7 +544,7 @@
     <col min="6" max="19" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="42" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -575,10 +596,10 @@
         <v>12</v>
       </c>
       <c r="H2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -620,7 +641,7 @@
         <v>21</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -629,25 +650,25 @@
         <v>1001</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G5" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="H5" s="2">
+      <c r="H5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I5" s="2">
         <v>0.8</v>
-      </c>
-      <c r="I5" s="2">
-        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="43" customHeight="1" x14ac:dyDescent="0.25">
@@ -656,25 +677,25 @@
         <v>1002</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="F6" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="G6" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="H6" s="2">
+        <v>26</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I6" s="2">
         <v>0.55000000000000004</v>
-      </c>
-      <c r="I6" s="2">
-        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="42.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -683,25 +704,25 @@
         <v>1003</v>
       </c>
       <c r="C7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="F7" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="G7" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="G7" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="H7" s="2">
+      <c r="H7" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I7" s="2">
         <v>0.25</v>
-      </c>
-      <c r="I7" s="2">
-        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add program office art assets
</commit_message>
<xml_diff>
--- a/Config/Luban/Datas/#game.gameEvent.xlsx
+++ b/Config/Luban/Datas/#game.gameEvent.xlsx
@@ -463,13 +463,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="4"/>
-    <col width="29.08984375" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="19"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -495,25 +495,35 @@
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
+          <t>yesText</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>noText</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
           <t>yesEffects#format=json</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>noEffects#format=json</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>triggerGreaterOrEqualConditions#format=json</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>triggerLessThanConditions#format=json</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>ratio</t>
         </is>
@@ -542,25 +552,35 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
           <t>array,array,int</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>array,array,int</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>array,array,int</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>array,array,int</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -580,6 +600,8 @@
       <c r="G3" s="2" t="n"/>
       <c r="H3" s="2" t="n"/>
       <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="n"/>
+      <c r="K3" s="2" t="n"/>
     </row>
     <row r="4" ht="93.5" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
@@ -604,25 +626,35 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
+          <t>选择文案</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>不选择文案</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
           <t>选择Y后的属性修改，格式[[属性ID,值]]</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>选择N后的属性修改，格式[[属性ID,值]]</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>大于等于触发条件，格式[[属性ID,阈值]]；玩家属性 &gt;= 阈值时满足</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>小于触发条件，格式[[属性ID,阈值]]；玩家属性 &lt; 阈值时满足</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Ratio（随机事件的触发概率）</t>
         </is>
@@ -639,30 +671,40 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>团队一早冒出一个大胆点子。选择 Y 立刻推进本周行动，选择 N 保守处理换一点预算。</t>
+          <t>团队一早冒出一个大胆点子。</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
+          <t>立刻推进本周行动</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>保守处理换一点预算</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
           <t>[[1002,1],[1009,6]]</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>[[1008,60]]</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>[[1005,30]]</t>
         </is>
       </c>
-      <c r="I5" s="2" t="n">
+      <c r="K5" s="2" t="n">
         <v>0.45</v>
       </c>
     </row>
@@ -677,30 +719,40 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>小型媒体提出本周试玩邀请。选择 Y 花钱打磨演示版换曝光，选择 N 推迟邀约。</t>
+          <t>小型媒体提出本周试玩邀请。</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
+          <t>花钱打磨演示版换曝光</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>推迟邀约</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
           <t>[[1008,-120],[1009,35],[1006,3],[1007,3]]</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>[[1008,60],[1009,-8]]</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>[[1009,30]]</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>[[1005,50]]</t>
         </is>
       </c>
-      <c r="I6" s="2" t="n">
+      <c r="K6" s="2" t="n">
         <v>0.35</v>
       </c>
     </row>
@@ -715,30 +767,40 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>一个顽固 Bug 被定位到了。选择 Y 消耗行动力集中修复，选择 N 暂时绕过问题。</t>
+          <t>一个顽固 Bug 被定位到了。</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
+          <t>消耗行动力集中修复</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>暂时绕过问题</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
           <t>[[1002,-1],[1005,-8],[1006,2],[1007,2]]</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>[[1005,4],[1008,80]]</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>[[1005,15]]</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="I7" s="2" t="n">
+      <c r="K7" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -753,30 +815,40 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>主视觉方案引发了分歧。选择 Y 坚持重做风格，选择 N 先用当前版本稳定进度。</t>
+          <t>主视觉方案引发了分歧。</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
+          <t>坚持重做风格</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>先用当前版本稳定进度</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
           <t>[[1006,12],[1005,3]]</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>[[1006,-4],[1009,5]]</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>[[1006,80]]</t>
         </is>
       </c>
-      <c r="I8" s="2" t="n">
+      <c r="K8" s="2" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -791,30 +863,40 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>外采音效出了版权小插曲。选择 Y 重新录制，选择 N 先替换成临时素材。</t>
+          <t>外采音效出了版权小插曲。</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
+          <t>重新录制</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>先替换成临时素材</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
           <t>[[1007,10],[1008,-80]]</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>[[1007,-5],[1005,2]]</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>[[1008,100]]</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="I9" s="2" t="n">
+      <c r="K9" s="2" t="n">
         <v>0.4</v>
       </c>
     </row>
@@ -829,30 +911,40 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>玩家社区自发传播了一张梗图。选择 Y 顺势运营，选择 N 低调观察热度。</t>
+          <t>玩家社区自发传播了一张梗图。</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
+          <t>顺势运营</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>低调观察热度</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
           <t>[[1009,40],[1024,5]]</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>[[1008,100],[1009,12]]</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>[[1006,30]]</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>[[1005,45]]</t>
         </is>
       </c>
-      <c r="I10" s="2" t="n">
+      <c r="K10" s="2" t="n">
         <v>0.3</v>
       </c>
     </row>
@@ -867,30 +959,40 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>可靠外包团队临时空出了档期。选择 Y 立刻签约补足产能，选择 N 留住现金流。</t>
+          <t>可靠外包团队临时空出了档期。</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
+          <t>立刻签约补足产能</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>留住现金流</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
           <t>[[1008,-180],[1029,4],[1030,4]]</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>[[1008,80]]</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>[[1008,250]]</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="I11" s="2" t="n">
+      <c r="K11" s="2" t="n">
         <v>0.38</v>
       </c>
     </row>
@@ -905,30 +1007,40 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>老版本里修过的问题又冒了出来。选择 Y 本周拉专项清掉，选择 N 先发布说明安抚。</t>
+          <t>老版本里修过的问题又冒了出来。</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
+          <t>本周拉专项清掉</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>先发布说明安抚</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
           <t>[[1005,-6],[1006,1],[1007,1]]</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>[[1005,10],[1009,-10]]</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>[[1005,20]]</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="I12" s="2" t="n">
+      <c r="K12" s="2" t="n">
         <v>0.6</v>
       </c>
     </row>
@@ -943,30 +1055,40 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>一位主播想提前试玩当前版本。选择 Y 提供内部包，选择 N 等稳定版本再联系。</t>
+          <t>一位主播想提前试玩当前版本。</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
+          <t>提供内部包</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>等稳定版本再联系</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
           <t>[[1008,-150],[1009,55],[1005,5]]</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>[[1008,80],[1009,10]]</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>[[1010,10]]</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>[[1005,35]]</t>
         </is>
       </c>
-      <c r="I13" s="2" t="n">
+      <c r="K13" s="2" t="n">
         <v>0.28</v>
       </c>
     </row>
@@ -981,30 +1103,40 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>连续赶工让团队有点疲惫。选择 Y 安排团建调整状态，选择 N 继续硬冲本周节点。</t>
+          <t>连续赶工让团队有点疲惫。</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
+          <t>安排团建调整状态</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>继续硬冲本周节点</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
           <t>[[1008,-100],[1006,6],[1007,8]]</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>[[1002,1],[1005,3]]</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>[[1009,100]]</t>
         </is>
       </c>
-      <c r="I14" s="2" t="n">
+      <c r="K14" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update game event data
</commit_message>
<xml_diff>
--- a/Config/Luban/Datas/#game.gameEvent.xlsx
+++ b/Config/Luban/Datas/#game.gameEvent.xlsx
@@ -728,7 +728,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>[[1008,-30000],[1005,-4]]</t>
+          <t>[[1008,-50000],[1005,-4]]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>[[1006,3]]</t>
+          <t>[[1008,-10000],[1006,5]]</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>[[1007,3]]</t>
+          <t>[[1008,-10000],[1007,5]]</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>[[1005,-5],[1006,-5]]</t>
+          <t>[[1006,-7],[1005,-5]]</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1218,12 +1218,12 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>[[1048,2],[1008,-50000]]</t>
+          <t>[[1008,-80000],[1048,2]]</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>[[1007,-2]]</t>
+          <t>[[1007,-5]]</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1316,12 +1316,12 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>[[1044,-1],[1005,-5]]</t>
+          <t>[[1005,-5],[1002,-2]]</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>[[1005,-1]]</t>
+          <t>[[1008,-10000],[1005,-3]]</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">

</xml_diff>